<commit_message>
Fixes issues with Fres
</commit_message>
<xml_diff>
--- a/data-raw/FOT_predictions_coefficient_tables_2024-02-16.xlsx
+++ b/data-raw/FOT_predictions_coefficient_tables_2024-02-16.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Principal_Investigators\Falvo\MATLAB SCRIPTS_Falvo\R_modules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tom/Documents/Positron/AHBPCE_Package/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E95579-8EB8-42AE-BDB4-CCF320AED56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB6CB28-E85D-8745-96B0-12784DA824CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{22FBC597-6A6E-4156-990A-E0A19A71570D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{22FBC597-6A6E-4156-990A-E0A19A71570D}"/>
   </bookViews>
   <sheets>
     <sheet name="Reactance" sheetId="1" r:id="rId1"/>
@@ -63,15 +63,6 @@
     <t>female_d</t>
   </si>
   <si>
-    <t>ln(fres)</t>
-  </si>
-  <si>
-    <t>ln(AX4)</t>
-  </si>
-  <si>
-    <t>ln(AX5)</t>
-  </si>
-  <si>
     <t>Frequency</t>
   </si>
   <si>
@@ -79,6 +70,15 @@
   </si>
   <si>
     <t>RSD_female</t>
+  </si>
+  <si>
+    <t>fres</t>
+  </si>
+  <si>
+    <t>AX5</t>
+  </si>
+  <si>
+    <t>AX4</t>
   </si>
 </sst>
 </file>
@@ -438,14 +438,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D2ED685-DC37-4E42-9202-EE2654A08B02}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -460,7 +460,7 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
         <v>3</v>
@@ -475,10 +475,10 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4</v>
       </c>
@@ -513,7 +513,7 @@
         <v>9.1800000000000007E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>5</v>
       </c>
@@ -548,7 +548,7 @@
         <v>8.14E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>6</v>
       </c>
@@ -583,7 +583,7 @@
         <v>8.0600000000000005E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>8</v>
       </c>
@@ -618,7 +618,7 @@
         <v>8.48E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>10</v>
       </c>
@@ -653,7 +653,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>12</v>
       </c>
@@ -688,7 +688,7 @@
         <v>9.9500000000000005E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>14</v>
       </c>
@@ -723,9 +723,9 @@
         <v>0.10879999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>5.07</v>
@@ -758,9 +758,9 @@
         <v>0.25490000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B10">
         <v>9.0340000000000007</v>
@@ -793,9 +793,9 @@
         <v>0.56730000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>9.73</v>
@@ -836,14 +836,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{671B3D8B-1F98-4546-BD8A-44655BCB425C}">
   <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -858,7 +858,7 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
         <v>3</v>
@@ -873,10 +873,10 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4</v>
       </c>
@@ -911,7 +911,7 @@
         <v>0.26369999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>5</v>
       </c>
@@ -946,7 +946,7 @@
         <v>0.26569999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>6</v>
       </c>
@@ -981,7 +981,7 @@
         <v>0.26479999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>7</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>0.26644999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>8</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>0.2681</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>10</v>
       </c>
@@ -1096,7 +1096,7 @@
         <v>0.26719999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>12</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>0.26369999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>14</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>0.25280000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>15</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>0.25619999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>16</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>0.24859999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>18</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>0.25219999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>19</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>0.24945000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>20</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>0.2467</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>22</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>0.25009999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>24</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>0.23830000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>26</v>
       </c>
@@ -1473,15 +1473,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004164715A01AFC6488ED70D61FA85B56C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d24d75978a3fe6b1358364101365183">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2651133f-d060-41ba-9146-7d56e4112d6e" xmlns:ns3="26378f15-1ba5-4d98-bde9-462191dd6aff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f96bebb32ee6bbfe7dacf57b0e2246b" ns2:_="" ns3:_="">
     <xsd:import namespace="2651133f-d060-41ba-9146-7d56e4112d6e"/>
@@ -1722,6 +1713,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{031E9264-E37D-4283-A183-02E3F7A7FFB1}">
   <ds:schemaRefs>
@@ -1734,14 +1734,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC23FE9-F6E4-48DC-9383-11E4CB4C2BC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00DB11BB-BA80-4616-855F-C5EEF804C27D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1758,4 +1750,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC23FE9-F6E4-48DC-9383-11E4CB4C2BC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>